<commit_message>
Add confirmation, reservation-form blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 20
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-confirmation.report.xlsx
+++ b/tools/importer/reports/import-confirmation.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="66">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,7 +61,7 @@
     <t>confirmation</t>
   </si>
   <si>
-    <t>2026-10-21T10:18:12.218Z</t>
+    <t>2026-10-23T10:26:27.467Z</t>
   </si>
   <si>
     <t>You're all set | JSW Motors</t>
@@ -76,7 +76,7 @@
     <t>confirmation.report.json</t>
   </si>
   <si>
-    <t>2026-10-21T10:18:07.139Z</t>
+    <t>2026-10-23T10:26:21.375Z</t>
   </si>
   <si>
     <t>Reserved | JSW Motors</t>
@@ -160,6 +160,21 @@
     <t>http://localhost:3000/drafts/new-energy/source.html</t>
   </si>
   <si>
+    <t>payment-failed.report.json</t>
+  </si>
+  <si>
+    <t>payment-failed</t>
+  </si>
+  <si>
+    <t>2026-10-23T10:26:33.521Z</t>
+  </si>
+  <si>
+    <t>Payment Failed | JSW Motors</t>
+  </si>
+  <si>
+    <t>http://localhost:3000/drafts/confirmation/source-payment-failed.html</t>
+  </si>
+  <si>
     <t>reservation-form.report.json</t>
   </si>
   <si>
@@ -169,7 +184,7 @@
     <t>reservation-form</t>
   </si>
   <si>
-    <t>2026-10-21T07:30:33.912Z</t>
+    <t>2026-10-23T10:26:17.068Z</t>
   </si>
   <si>
     <t>Reserve Now | JSW Motors</t>
@@ -582,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -856,10 +871,10 @@
         <v>49</v>
       </c>
       <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
         <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>51</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
@@ -868,30 +883,30 @@
         <v>14</v>
       </c>
       <c r="F9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
         <v>51</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>52</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>53</v>
       </c>
-      <c r="I9" t="s">
-        <v>54</v>
-      </c>
       <c r="J9" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>56</v>
-      </c>
-      <c r="C10" t="s">
-        <v>57</v>
       </c>
       <c r="D10" t="s">
         <v>13</v>
@@ -900,18 +915,50 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
         <v>57</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>58</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>59</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>60</v>
       </c>
-      <c r="J10" t="s">
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" t="s">
+        <v>63</v>
+      </c>
+      <c r="H11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>